<commit_message>
change growth of $10,000 to show final value
</commit_message>
<xml_diff>
--- a/data/fmc.xlsx
+++ b/data/fmc.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6113f60f932799a7/1Evan/.eff_fron_spyder/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{EE1D38D0-8CE8-4AD8-990B-3B50A5A5D4AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF33CAAE-8380-48DE-B0E9-5F1CCC521EE6}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{EE1D38D0-8CE8-4AD8-990B-3B50A5A5D4AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2A25EB4-E21A-42BE-9C20-9BBDB552490E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investments" sheetId="1" r:id="rId1"/>
-    <sheet name="Dates &amp;amp;amp;amp;amp;amp; Ris" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,16 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>End Date</t>
-  </si>
-  <si>
-    <t>Risk Free Rate</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Ticker</t>
   </si>
@@ -113,8 +103,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.00%"/>
-    <numFmt numFmtId="165" formatCode="#,##0%"/>
+    <numFmt numFmtId="164" formatCode="#,##0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -158,39 +148,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,262 +471,275 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.453125" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="8">
-        <v>0</v>
-      </c>
-      <c r="C2" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="8">
-        <v>0</v>
-      </c>
-      <c r="C3" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="8">
-        <v>0</v>
-      </c>
-      <c r="C4" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="8">
-        <v>0</v>
-      </c>
-      <c r="C5" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="8">
-        <v>0</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="8">
-        <v>0</v>
-      </c>
-      <c r="C8" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="8">
-        <v>0</v>
-      </c>
-      <c r="C9" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="8">
-        <v>0</v>
-      </c>
-      <c r="C10" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="8">
-        <v>0</v>
-      </c>
-      <c r="C11" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="8">
-        <v>0</v>
-      </c>
-      <c r="C12" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="8">
-        <v>0</v>
-      </c>
-      <c r="C13" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="8">
-        <v>0</v>
-      </c>
-      <c r="C14" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="8">
-        <v>0</v>
-      </c>
-      <c r="C15" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="8">
-        <v>0</v>
-      </c>
-      <c r="C16" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="8">
-        <v>0</v>
-      </c>
-      <c r="C17" s="8">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="8">
-        <v>0</v>
-      </c>
-      <c r="C18" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="8">
-        <v>0</v>
-      </c>
-      <c r="C19" s="8">
-        <v>0.1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="2" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" style="6" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
-        <f ca="1">DATE(YEAR(B2)-10,MONTH(B2),DAY(B2))</f>
-        <v>41859</v>
-      </c>
-      <c r="B2" s="3">
-        <f ca="1">NOW()</f>
-        <v>45512.544621064815</v>
-      </c>
-      <c r="C2" s="4">
-        <v>5.1499999999999997E-2</v>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="2">
+        <v>0</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.99999000000000005</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>